<commit_message>
feat: remove all preloaded student data, provide clean intake template, and clean empty state
</commit_message>
<xml_diff>
--- a/public/samples/Hanyang-Student-Intake-Template.xlsx
+++ b/public/samples/Hanyang-Student-Intake-Template.xlsx
@@ -76,16 +76,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -453,7 +450,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J29"/>
+  <dimension ref="A1:J51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -520,465 +517,705 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="22" customHeight="1">
+    <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>2025832474</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>MINAN MD ABDULLAH AL</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>2003-06-15</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="inlineStr">
-        <is>
-          <t>Korean Language Course</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>Bachelor of Business Administration</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>2025-12-03</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>2026-12-12</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>2025-10-01</t>
-        </is>
-      </c>
-      <c r="J2" s="3" t="inlineStr">
-        <is>
-          <t>Sample record (can be overwritten or deleted)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="22" customHeight="1">
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="3" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="3" t="n"/>
+      <c r="F2" s="3" t="n"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="2" t="n"/>
+      <c r="J2" s="3" t="n"/>
+    </row>
+    <row r="3" ht="20" customHeight="1">
       <c r="A3" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>2026832423</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>CHAKMA PRATIK</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>2006-02-08</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>Korean Language Course</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>Bachelor of Business Administration</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>2026-12-02</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>2027-02-12</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-06</t>
-        </is>
-      </c>
-      <c r="J3" s="3" t="inlineStr"/>
+      <c r="B3" s="2" t="n"/>
+      <c r="C3" s="3" t="n"/>
+      <c r="D3" s="2" t="n"/>
+      <c r="E3" s="3" t="n"/>
+      <c r="F3" s="3" t="n"/>
+      <c r="G3" s="2" t="n"/>
+      <c r="H3" s="2" t="n"/>
+      <c r="I3" s="2" t="n"/>
+      <c r="J3" s="3" t="n"/>
     </row>
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="2" t="n">
         <v>3</v>
       </c>
       <c r="B4" s="2" t="n"/>
-      <c r="C4" s="4" t="n"/>
+      <c r="C4" s="3" t="n"/>
       <c r="D4" s="2" t="n"/>
-      <c r="E4" s="4" t="n"/>
-      <c r="F4" s="4" t="n"/>
+      <c r="E4" s="3" t="n"/>
+      <c r="F4" s="3" t="n"/>
       <c r="G4" s="2" t="n"/>
       <c r="H4" s="2" t="n"/>
       <c r="I4" s="2" t="n"/>
-      <c r="J4" s="4" t="n"/>
+      <c r="J4" s="3" t="n"/>
     </row>
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="2" t="n">
         <v>4</v>
       </c>
       <c r="B5" s="2" t="n"/>
-      <c r="C5" s="4" t="n"/>
+      <c r="C5" s="3" t="n"/>
       <c r="D5" s="2" t="n"/>
-      <c r="E5" s="4" t="n"/>
-      <c r="F5" s="4" t="n"/>
+      <c r="E5" s="3" t="n"/>
+      <c r="F5" s="3" t="n"/>
       <c r="G5" s="2" t="n"/>
       <c r="H5" s="2" t="n"/>
       <c r="I5" s="2" t="n"/>
-      <c r="J5" s="4" t="n"/>
+      <c r="J5" s="3" t="n"/>
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="2" t="n">
         <v>5</v>
       </c>
       <c r="B6" s="2" t="n"/>
-      <c r="C6" s="4" t="n"/>
+      <c r="C6" s="3" t="n"/>
       <c r="D6" s="2" t="n"/>
-      <c r="E6" s="4" t="n"/>
-      <c r="F6" s="4" t="n"/>
+      <c r="E6" s="3" t="n"/>
+      <c r="F6" s="3" t="n"/>
       <c r="G6" s="2" t="n"/>
       <c r="H6" s="2" t="n"/>
       <c r="I6" s="2" t="n"/>
-      <c r="J6" s="4" t="n"/>
+      <c r="J6" s="3" t="n"/>
     </row>
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="2" t="n">
         <v>6</v>
       </c>
       <c r="B7" s="2" t="n"/>
-      <c r="C7" s="4" t="n"/>
+      <c r="C7" s="3" t="n"/>
       <c r="D7" s="2" t="n"/>
-      <c r="E7" s="4" t="n"/>
-      <c r="F7" s="4" t="n"/>
+      <c r="E7" s="3" t="n"/>
+      <c r="F7" s="3" t="n"/>
       <c r="G7" s="2" t="n"/>
       <c r="H7" s="2" t="n"/>
       <c r="I7" s="2" t="n"/>
-      <c r="J7" s="4" t="n"/>
+      <c r="J7" s="3" t="n"/>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="2" t="n">
         <v>7</v>
       </c>
       <c r="B8" s="2" t="n"/>
-      <c r="C8" s="4" t="n"/>
+      <c r="C8" s="3" t="n"/>
       <c r="D8" s="2" t="n"/>
-      <c r="E8" s="4" t="n"/>
-      <c r="F8" s="4" t="n"/>
+      <c r="E8" s="3" t="n"/>
+      <c r="F8" s="3" t="n"/>
       <c r="G8" s="2" t="n"/>
       <c r="H8" s="2" t="n"/>
       <c r="I8" s="2" t="n"/>
-      <c r="J8" s="4" t="n"/>
+      <c r="J8" s="3" t="n"/>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="2" t="n">
         <v>8</v>
       </c>
       <c r="B9" s="2" t="n"/>
-      <c r="C9" s="4" t="n"/>
+      <c r="C9" s="3" t="n"/>
       <c r="D9" s="2" t="n"/>
-      <c r="E9" s="4" t="n"/>
-      <c r="F9" s="4" t="n"/>
+      <c r="E9" s="3" t="n"/>
+      <c r="F9" s="3" t="n"/>
       <c r="G9" s="2" t="n"/>
       <c r="H9" s="2" t="n"/>
       <c r="I9" s="2" t="n"/>
-      <c r="J9" s="4" t="n"/>
+      <c r="J9" s="3" t="n"/>
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="2" t="n">
         <v>9</v>
       </c>
       <c r="B10" s="2" t="n"/>
-      <c r="C10" s="4" t="n"/>
+      <c r="C10" s="3" t="n"/>
       <c r="D10" s="2" t="n"/>
-      <c r="E10" s="4" t="n"/>
-      <c r="F10" s="4" t="n"/>
+      <c r="E10" s="3" t="n"/>
+      <c r="F10" s="3" t="n"/>
       <c r="G10" s="2" t="n"/>
       <c r="H10" s="2" t="n"/>
       <c r="I10" s="2" t="n"/>
-      <c r="J10" s="4" t="n"/>
+      <c r="J10" s="3" t="n"/>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="2" t="n">
         <v>10</v>
       </c>
       <c r="B11" s="2" t="n"/>
-      <c r="C11" s="4" t="n"/>
+      <c r="C11" s="3" t="n"/>
       <c r="D11" s="2" t="n"/>
-      <c r="E11" s="4" t="n"/>
-      <c r="F11" s="4" t="n"/>
+      <c r="E11" s="3" t="n"/>
+      <c r="F11" s="3" t="n"/>
       <c r="G11" s="2" t="n"/>
       <c r="H11" s="2" t="n"/>
       <c r="I11" s="2" t="n"/>
-      <c r="J11" s="4" t="n"/>
+      <c r="J11" s="3" t="n"/>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="2" t="n">
         <v>11</v>
       </c>
       <c r="B12" s="2" t="n"/>
-      <c r="C12" s="4" t="n"/>
+      <c r="C12" s="3" t="n"/>
       <c r="D12" s="2" t="n"/>
-      <c r="E12" s="4" t="n"/>
-      <c r="F12" s="4" t="n"/>
+      <c r="E12" s="3" t="n"/>
+      <c r="F12" s="3" t="n"/>
       <c r="G12" s="2" t="n"/>
       <c r="H12" s="2" t="n"/>
       <c r="I12" s="2" t="n"/>
-      <c r="J12" s="4" t="n"/>
+      <c r="J12" s="3" t="n"/>
     </row>
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="2" t="n">
         <v>12</v>
       </c>
       <c r="B13" s="2" t="n"/>
-      <c r="C13" s="4" t="n"/>
+      <c r="C13" s="3" t="n"/>
       <c r="D13" s="2" t="n"/>
-      <c r="E13" s="4" t="n"/>
-      <c r="F13" s="4" t="n"/>
+      <c r="E13" s="3" t="n"/>
+      <c r="F13" s="3" t="n"/>
       <c r="G13" s="2" t="n"/>
       <c r="H13" s="2" t="n"/>
       <c r="I13" s="2" t="n"/>
-      <c r="J13" s="4" t="n"/>
+      <c r="J13" s="3" t="n"/>
     </row>
     <row r="14" ht="20" customHeight="1">
       <c r="A14" s="2" t="n">
         <v>13</v>
       </c>
       <c r="B14" s="2" t="n"/>
-      <c r="C14" s="4" t="n"/>
+      <c r="C14" s="3" t="n"/>
       <c r="D14" s="2" t="n"/>
-      <c r="E14" s="4" t="n"/>
-      <c r="F14" s="4" t="n"/>
+      <c r="E14" s="3" t="n"/>
+      <c r="F14" s="3" t="n"/>
       <c r="G14" s="2" t="n"/>
       <c r="H14" s="2" t="n"/>
       <c r="I14" s="2" t="n"/>
-      <c r="J14" s="4" t="n"/>
+      <c r="J14" s="3" t="n"/>
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="2" t="n">
         <v>14</v>
       </c>
       <c r="B15" s="2" t="n"/>
-      <c r="C15" s="4" t="n"/>
+      <c r="C15" s="3" t="n"/>
       <c r="D15" s="2" t="n"/>
-      <c r="E15" s="4" t="n"/>
-      <c r="F15" s="4" t="n"/>
+      <c r="E15" s="3" t="n"/>
+      <c r="F15" s="3" t="n"/>
       <c r="G15" s="2" t="n"/>
       <c r="H15" s="2" t="n"/>
       <c r="I15" s="2" t="n"/>
-      <c r="J15" s="4" t="n"/>
+      <c r="J15" s="3" t="n"/>
     </row>
     <row r="16" ht="20" customHeight="1">
       <c r="A16" s="2" t="n">
         <v>15</v>
       </c>
       <c r="B16" s="2" t="n"/>
-      <c r="C16" s="4" t="n"/>
+      <c r="C16" s="3" t="n"/>
       <c r="D16" s="2" t="n"/>
-      <c r="E16" s="4" t="n"/>
-      <c r="F16" s="4" t="n"/>
+      <c r="E16" s="3" t="n"/>
+      <c r="F16" s="3" t="n"/>
       <c r="G16" s="2" t="n"/>
       <c r="H16" s="2" t="n"/>
       <c r="I16" s="2" t="n"/>
-      <c r="J16" s="4" t="n"/>
+      <c r="J16" s="3" t="n"/>
     </row>
     <row r="17" ht="20" customHeight="1">
       <c r="A17" s="2" t="n">
         <v>16</v>
       </c>
       <c r="B17" s="2" t="n"/>
-      <c r="C17" s="4" t="n"/>
+      <c r="C17" s="3" t="n"/>
       <c r="D17" s="2" t="n"/>
-      <c r="E17" s="4" t="n"/>
-      <c r="F17" s="4" t="n"/>
+      <c r="E17" s="3" t="n"/>
+      <c r="F17" s="3" t="n"/>
       <c r="G17" s="2" t="n"/>
       <c r="H17" s="2" t="n"/>
       <c r="I17" s="2" t="n"/>
-      <c r="J17" s="4" t="n"/>
+      <c r="J17" s="3" t="n"/>
     </row>
     <row r="18" ht="20" customHeight="1">
       <c r="A18" s="2" t="n">
         <v>17</v>
       </c>
       <c r="B18" s="2" t="n"/>
-      <c r="C18" s="4" t="n"/>
+      <c r="C18" s="3" t="n"/>
       <c r="D18" s="2" t="n"/>
-      <c r="E18" s="4" t="n"/>
-      <c r="F18" s="4" t="n"/>
+      <c r="E18" s="3" t="n"/>
+      <c r="F18" s="3" t="n"/>
       <c r="G18" s="2" t="n"/>
       <c r="H18" s="2" t="n"/>
       <c r="I18" s="2" t="n"/>
-      <c r="J18" s="4" t="n"/>
+      <c r="J18" s="3" t="n"/>
     </row>
     <row r="19" ht="20" customHeight="1">
       <c r="A19" s="2" t="n">
         <v>18</v>
       </c>
       <c r="B19" s="2" t="n"/>
-      <c r="C19" s="4" t="n"/>
+      <c r="C19" s="3" t="n"/>
       <c r="D19" s="2" t="n"/>
-      <c r="E19" s="4" t="n"/>
-      <c r="F19" s="4" t="n"/>
+      <c r="E19" s="3" t="n"/>
+      <c r="F19" s="3" t="n"/>
       <c r="G19" s="2" t="n"/>
       <c r="H19" s="2" t="n"/>
       <c r="I19" s="2" t="n"/>
-      <c r="J19" s="4" t="n"/>
+      <c r="J19" s="3" t="n"/>
     </row>
     <row r="20" ht="20" customHeight="1">
       <c r="A20" s="2" t="n">
         <v>19</v>
       </c>
       <c r="B20" s="2" t="n"/>
-      <c r="C20" s="4" t="n"/>
+      <c r="C20" s="3" t="n"/>
       <c r="D20" s="2" t="n"/>
-      <c r="E20" s="4" t="n"/>
-      <c r="F20" s="4" t="n"/>
+      <c r="E20" s="3" t="n"/>
+      <c r="F20" s="3" t="n"/>
       <c r="G20" s="2" t="n"/>
       <c r="H20" s="2" t="n"/>
       <c r="I20" s="2" t="n"/>
-      <c r="J20" s="4" t="n"/>
+      <c r="J20" s="3" t="n"/>
     </row>
     <row r="21" ht="20" customHeight="1">
       <c r="A21" s="2" t="n">
         <v>20</v>
       </c>
       <c r="B21" s="2" t="n"/>
-      <c r="C21" s="4" t="n"/>
+      <c r="C21" s="3" t="n"/>
       <c r="D21" s="2" t="n"/>
-      <c r="E21" s="4" t="n"/>
-      <c r="F21" s="4" t="n"/>
+      <c r="E21" s="3" t="n"/>
+      <c r="F21" s="3" t="n"/>
       <c r="G21" s="2" t="n"/>
       <c r="H21" s="2" t="n"/>
       <c r="I21" s="2" t="n"/>
-      <c r="J21" s="4" t="n"/>
+      <c r="J21" s="3" t="n"/>
     </row>
     <row r="22" ht="20" customHeight="1">
       <c r="A22" s="2" t="n">
         <v>21</v>
       </c>
       <c r="B22" s="2" t="n"/>
-      <c r="C22" s="4" t="n"/>
+      <c r="C22" s="3" t="n"/>
       <c r="D22" s="2" t="n"/>
-      <c r="E22" s="4" t="n"/>
-      <c r="F22" s="4" t="n"/>
+      <c r="E22" s="3" t="n"/>
+      <c r="F22" s="3" t="n"/>
       <c r="G22" s="2" t="n"/>
       <c r="H22" s="2" t="n"/>
       <c r="I22" s="2" t="n"/>
-      <c r="J22" s="4" t="n"/>
+      <c r="J22" s="3" t="n"/>
     </row>
     <row r="23" ht="20" customHeight="1">
       <c r="A23" s="2" t="n">
         <v>22</v>
       </c>
       <c r="B23" s="2" t="n"/>
-      <c r="C23" s="4" t="n"/>
+      <c r="C23" s="3" t="n"/>
       <c r="D23" s="2" t="n"/>
-      <c r="E23" s="4" t="n"/>
-      <c r="F23" s="4" t="n"/>
+      <c r="E23" s="3" t="n"/>
+      <c r="F23" s="3" t="n"/>
       <c r="G23" s="2" t="n"/>
       <c r="H23" s="2" t="n"/>
       <c r="I23" s="2" t="n"/>
-      <c r="J23" s="4" t="n"/>
+      <c r="J23" s="3" t="n"/>
     </row>
     <row r="24" ht="20" customHeight="1">
       <c r="A24" s="2" t="n">
         <v>23</v>
       </c>
       <c r="B24" s="2" t="n"/>
-      <c r="C24" s="4" t="n"/>
+      <c r="C24" s="3" t="n"/>
       <c r="D24" s="2" t="n"/>
-      <c r="E24" s="4" t="n"/>
-      <c r="F24" s="4" t="n"/>
+      <c r="E24" s="3" t="n"/>
+      <c r="F24" s="3" t="n"/>
       <c r="G24" s="2" t="n"/>
       <c r="H24" s="2" t="n"/>
       <c r="I24" s="2" t="n"/>
-      <c r="J24" s="4" t="n"/>
+      <c r="J24" s="3" t="n"/>
     </row>
     <row r="25" ht="20" customHeight="1">
       <c r="A25" s="2" t="n">
         <v>24</v>
       </c>
       <c r="B25" s="2" t="n"/>
-      <c r="C25" s="4" t="n"/>
+      <c r="C25" s="3" t="n"/>
       <c r="D25" s="2" t="n"/>
-      <c r="E25" s="4" t="n"/>
-      <c r="F25" s="4" t="n"/>
+      <c r="E25" s="3" t="n"/>
+      <c r="F25" s="3" t="n"/>
       <c r="G25" s="2" t="n"/>
       <c r="H25" s="2" t="n"/>
       <c r="I25" s="2" t="n"/>
-      <c r="J25" s="4" t="n"/>
+      <c r="J25" s="3" t="n"/>
     </row>
     <row r="26" ht="20" customHeight="1">
       <c r="A26" s="2" t="n">
         <v>25</v>
       </c>
       <c r="B26" s="2" t="n"/>
-      <c r="C26" s="4" t="n"/>
+      <c r="C26" s="3" t="n"/>
       <c r="D26" s="2" t="n"/>
-      <c r="E26" s="4" t="n"/>
-      <c r="F26" s="4" t="n"/>
+      <c r="E26" s="3" t="n"/>
+      <c r="F26" s="3" t="n"/>
       <c r="G26" s="2" t="n"/>
       <c r="H26" s="2" t="n"/>
       <c r="I26" s="2" t="n"/>
-      <c r="J26" s="4" t="n"/>
+      <c r="J26" s="3" t="n"/>
     </row>
     <row r="27" ht="20" customHeight="1">
       <c r="A27" s="2" t="n">
         <v>26</v>
       </c>
       <c r="B27" s="2" t="n"/>
-      <c r="C27" s="4" t="n"/>
+      <c r="C27" s="3" t="n"/>
       <c r="D27" s="2" t="n"/>
-      <c r="E27" s="4" t="n"/>
-      <c r="F27" s="4" t="n"/>
+      <c r="E27" s="3" t="n"/>
+      <c r="F27" s="3" t="n"/>
       <c r="G27" s="2" t="n"/>
       <c r="H27" s="2" t="n"/>
       <c r="I27" s="2" t="n"/>
-      <c r="J27" s="4" t="n"/>
+      <c r="J27" s="3" t="n"/>
     </row>
     <row r="28" ht="20" customHeight="1">
       <c r="A28" s="2" t="n">
         <v>27</v>
       </c>
       <c r="B28" s="2" t="n"/>
-      <c r="C28" s="4" t="n"/>
+      <c r="C28" s="3" t="n"/>
       <c r="D28" s="2" t="n"/>
-      <c r="E28" s="4" t="n"/>
-      <c r="F28" s="4" t="n"/>
+      <c r="E28" s="3" t="n"/>
+      <c r="F28" s="3" t="n"/>
       <c r="G28" s="2" t="n"/>
       <c r="H28" s="2" t="n"/>
       <c r="I28" s="2" t="n"/>
-      <c r="J28" s="4" t="n"/>
+      <c r="J28" s="3" t="n"/>
     </row>
     <row r="29" ht="20" customHeight="1">
       <c r="A29" s="2" t="n">
         <v>28</v>
       </c>
       <c r="B29" s="2" t="n"/>
-      <c r="C29" s="4" t="n"/>
+      <c r="C29" s="3" t="n"/>
       <c r="D29" s="2" t="n"/>
-      <c r="E29" s="4" t="n"/>
-      <c r="F29" s="4" t="n"/>
+      <c r="E29" s="3" t="n"/>
+      <c r="F29" s="3" t="n"/>
       <c r="G29" s="2" t="n"/>
       <c r="H29" s="2" t="n"/>
       <c r="I29" s="2" t="n"/>
-      <c r="J29" s="4" t="n"/>
+      <c r="J29" s="3" t="n"/>
+    </row>
+    <row r="30" ht="20" customHeight="1">
+      <c r="A30" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="2" t="n"/>
+      <c r="C30" s="3" t="n"/>
+      <c r="D30" s="2" t="n"/>
+      <c r="E30" s="3" t="n"/>
+      <c r="F30" s="3" t="n"/>
+      <c r="G30" s="2" t="n"/>
+      <c r="H30" s="2" t="n"/>
+      <c r="I30" s="2" t="n"/>
+      <c r="J30" s="3" t="n"/>
+    </row>
+    <row r="31" ht="20" customHeight="1">
+      <c r="A31" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="2" t="n"/>
+      <c r="C31" s="3" t="n"/>
+      <c r="D31" s="2" t="n"/>
+      <c r="E31" s="3" t="n"/>
+      <c r="F31" s="3" t="n"/>
+      <c r="G31" s="2" t="n"/>
+      <c r="H31" s="2" t="n"/>
+      <c r="I31" s="2" t="n"/>
+      <c r="J31" s="3" t="n"/>
+    </row>
+    <row r="32" ht="20" customHeight="1">
+      <c r="A32" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="2" t="n"/>
+      <c r="C32" s="3" t="n"/>
+      <c r="D32" s="2" t="n"/>
+      <c r="E32" s="3" t="n"/>
+      <c r="F32" s="3" t="n"/>
+      <c r="G32" s="2" t="n"/>
+      <c r="H32" s="2" t="n"/>
+      <c r="I32" s="2" t="n"/>
+      <c r="J32" s="3" t="n"/>
+    </row>
+    <row r="33" ht="20" customHeight="1">
+      <c r="A33" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="2" t="n"/>
+      <c r="C33" s="3" t="n"/>
+      <c r="D33" s="2" t="n"/>
+      <c r="E33" s="3" t="n"/>
+      <c r="F33" s="3" t="n"/>
+      <c r="G33" s="2" t="n"/>
+      <c r="H33" s="2" t="n"/>
+      <c r="I33" s="2" t="n"/>
+      <c r="J33" s="3" t="n"/>
+    </row>
+    <row r="34" ht="20" customHeight="1">
+      <c r="A34" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="2" t="n"/>
+      <c r="C34" s="3" t="n"/>
+      <c r="D34" s="2" t="n"/>
+      <c r="E34" s="3" t="n"/>
+      <c r="F34" s="3" t="n"/>
+      <c r="G34" s="2" t="n"/>
+      <c r="H34" s="2" t="n"/>
+      <c r="I34" s="2" t="n"/>
+      <c r="J34" s="3" t="n"/>
+    </row>
+    <row r="35" ht="20" customHeight="1">
+      <c r="A35" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="2" t="n"/>
+      <c r="C35" s="3" t="n"/>
+      <c r="D35" s="2" t="n"/>
+      <c r="E35" s="3" t="n"/>
+      <c r="F35" s="3" t="n"/>
+      <c r="G35" s="2" t="n"/>
+      <c r="H35" s="2" t="n"/>
+      <c r="I35" s="2" t="n"/>
+      <c r="J35" s="3" t="n"/>
+    </row>
+    <row r="36" ht="20" customHeight="1">
+      <c r="A36" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="2" t="n"/>
+      <c r="C36" s="3" t="n"/>
+      <c r="D36" s="2" t="n"/>
+      <c r="E36" s="3" t="n"/>
+      <c r="F36" s="3" t="n"/>
+      <c r="G36" s="2" t="n"/>
+      <c r="H36" s="2" t="n"/>
+      <c r="I36" s="2" t="n"/>
+      <c r="J36" s="3" t="n"/>
+    </row>
+    <row r="37" ht="20" customHeight="1">
+      <c r="A37" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="2" t="n"/>
+      <c r="C37" s="3" t="n"/>
+      <c r="D37" s="2" t="n"/>
+      <c r="E37" s="3" t="n"/>
+      <c r="F37" s="3" t="n"/>
+      <c r="G37" s="2" t="n"/>
+      <c r="H37" s="2" t="n"/>
+      <c r="I37" s="2" t="n"/>
+      <c r="J37" s="3" t="n"/>
+    </row>
+    <row r="38" ht="20" customHeight="1">
+      <c r="A38" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="2" t="n"/>
+      <c r="C38" s="3" t="n"/>
+      <c r="D38" s="2" t="n"/>
+      <c r="E38" s="3" t="n"/>
+      <c r="F38" s="3" t="n"/>
+      <c r="G38" s="2" t="n"/>
+      <c r="H38" s="2" t="n"/>
+      <c r="I38" s="2" t="n"/>
+      <c r="J38" s="3" t="n"/>
+    </row>
+    <row r="39" ht="20" customHeight="1">
+      <c r="A39" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="2" t="n"/>
+      <c r="C39" s="3" t="n"/>
+      <c r="D39" s="2" t="n"/>
+      <c r="E39" s="3" t="n"/>
+      <c r="F39" s="3" t="n"/>
+      <c r="G39" s="2" t="n"/>
+      <c r="H39" s="2" t="n"/>
+      <c r="I39" s="2" t="n"/>
+      <c r="J39" s="3" t="n"/>
+    </row>
+    <row r="40" ht="20" customHeight="1">
+      <c r="A40" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="2" t="n"/>
+      <c r="C40" s="3" t="n"/>
+      <c r="D40" s="2" t="n"/>
+      <c r="E40" s="3" t="n"/>
+      <c r="F40" s="3" t="n"/>
+      <c r="G40" s="2" t="n"/>
+      <c r="H40" s="2" t="n"/>
+      <c r="I40" s="2" t="n"/>
+      <c r="J40" s="3" t="n"/>
+    </row>
+    <row r="41" ht="20" customHeight="1">
+      <c r="A41" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="2" t="n"/>
+      <c r="C41" s="3" t="n"/>
+      <c r="D41" s="2" t="n"/>
+      <c r="E41" s="3" t="n"/>
+      <c r="F41" s="3" t="n"/>
+      <c r="G41" s="2" t="n"/>
+      <c r="H41" s="2" t="n"/>
+      <c r="I41" s="2" t="n"/>
+      <c r="J41" s="3" t="n"/>
+    </row>
+    <row r="42" ht="20" customHeight="1">
+      <c r="A42" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="2" t="n"/>
+      <c r="C42" s="3" t="n"/>
+      <c r="D42" s="2" t="n"/>
+      <c r="E42" s="3" t="n"/>
+      <c r="F42" s="3" t="n"/>
+      <c r="G42" s="2" t="n"/>
+      <c r="H42" s="2" t="n"/>
+      <c r="I42" s="2" t="n"/>
+      <c r="J42" s="3" t="n"/>
+    </row>
+    <row r="43" ht="20" customHeight="1">
+      <c r="A43" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="2" t="n"/>
+      <c r="C43" s="3" t="n"/>
+      <c r="D43" s="2" t="n"/>
+      <c r="E43" s="3" t="n"/>
+      <c r="F43" s="3" t="n"/>
+      <c r="G43" s="2" t="n"/>
+      <c r="H43" s="2" t="n"/>
+      <c r="I43" s="2" t="n"/>
+      <c r="J43" s="3" t="n"/>
+    </row>
+    <row r="44" ht="20" customHeight="1">
+      <c r="A44" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="2" t="n"/>
+      <c r="C44" s="3" t="n"/>
+      <c r="D44" s="2" t="n"/>
+      <c r="E44" s="3" t="n"/>
+      <c r="F44" s="3" t="n"/>
+      <c r="G44" s="2" t="n"/>
+      <c r="H44" s="2" t="n"/>
+      <c r="I44" s="2" t="n"/>
+      <c r="J44" s="3" t="n"/>
+    </row>
+    <row r="45" ht="20" customHeight="1">
+      <c r="A45" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="2" t="n"/>
+      <c r="C45" s="3" t="n"/>
+      <c r="D45" s="2" t="n"/>
+      <c r="E45" s="3" t="n"/>
+      <c r="F45" s="3" t="n"/>
+      <c r="G45" s="2" t="n"/>
+      <c r="H45" s="2" t="n"/>
+      <c r="I45" s="2" t="n"/>
+      <c r="J45" s="3" t="n"/>
+    </row>
+    <row r="46" ht="20" customHeight="1">
+      <c r="A46" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="2" t="n"/>
+      <c r="C46" s="3" t="n"/>
+      <c r="D46" s="2" t="n"/>
+      <c r="E46" s="3" t="n"/>
+      <c r="F46" s="3" t="n"/>
+      <c r="G46" s="2" t="n"/>
+      <c r="H46" s="2" t="n"/>
+      <c r="I46" s="2" t="n"/>
+      <c r="J46" s="3" t="n"/>
+    </row>
+    <row r="47" ht="20" customHeight="1">
+      <c r="A47" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="2" t="n"/>
+      <c r="C47" s="3" t="n"/>
+      <c r="D47" s="2" t="n"/>
+      <c r="E47" s="3" t="n"/>
+      <c r="F47" s="3" t="n"/>
+      <c r="G47" s="2" t="n"/>
+      <c r="H47" s="2" t="n"/>
+      <c r="I47" s="2" t="n"/>
+      <c r="J47" s="3" t="n"/>
+    </row>
+    <row r="48" ht="20" customHeight="1">
+      <c r="A48" s="2" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="2" t="n"/>
+      <c r="C48" s="3" t="n"/>
+      <c r="D48" s="2" t="n"/>
+      <c r="E48" s="3" t="n"/>
+      <c r="F48" s="3" t="n"/>
+      <c r="G48" s="2" t="n"/>
+      <c r="H48" s="2" t="n"/>
+      <c r="I48" s="2" t="n"/>
+      <c r="J48" s="3" t="n"/>
+    </row>
+    <row r="49" ht="20" customHeight="1">
+      <c r="A49" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="2" t="n"/>
+      <c r="C49" s="3" t="n"/>
+      <c r="D49" s="2" t="n"/>
+      <c r="E49" s="3" t="n"/>
+      <c r="F49" s="3" t="n"/>
+      <c r="G49" s="2" t="n"/>
+      <c r="H49" s="2" t="n"/>
+      <c r="I49" s="2" t="n"/>
+      <c r="J49" s="3" t="n"/>
+    </row>
+    <row r="50" ht="20" customHeight="1">
+      <c r="A50" s="2" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="2" t="n"/>
+      <c r="C50" s="3" t="n"/>
+      <c r="D50" s="2" t="n"/>
+      <c r="E50" s="3" t="n"/>
+      <c r="F50" s="3" t="n"/>
+      <c r="G50" s="2" t="n"/>
+      <c r="H50" s="2" t="n"/>
+      <c r="I50" s="2" t="n"/>
+      <c r="J50" s="3" t="n"/>
+    </row>
+    <row r="51" ht="20" customHeight="1">
+      <c r="A51" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="2" t="n"/>
+      <c r="C51" s="3" t="n"/>
+      <c r="D51" s="2" t="n"/>
+      <c r="E51" s="3" t="n"/>
+      <c r="F51" s="3" t="n"/>
+      <c r="G51" s="2" t="n"/>
+      <c r="H51" s="2" t="n"/>
+      <c r="I51" s="2" t="n"/>
+      <c r="J51" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>